<commit_message>
Doing some fun work, it has to be fun you rmember???
</commit_message>
<xml_diff>
--- a/oversikt.xlsx
+++ b/oversikt.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="32">
   <si>
     <t xml:space="preserve">Uke</t>
   </si>
@@ -73,25 +73,16 @@
     <t xml:space="preserve">Discrete-time signals and systems</t>
   </si>
   <si>
-    <t xml:space="preserve">x (70%)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Z-transform</t>
   </si>
   <si>
-    <t xml:space="preserve">x (30%)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Fourier representation of signal</t>
   </si>
   <si>
-    <t xml:space="preserve">x (20%)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Skipper denne nå for å henge
-Med I forelesning.
-Dette kan jeg tross alt ganske bra.
-Kan komme tilbake til dette.</t>
+    <t xml:space="preserve">X (80%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Du kan evt. gjøre oppgave 3 for å se på DTFT egenskaper.</t>
   </si>
   <si>
     <t xml:space="preserve">Introduction to project</t>
@@ -118,6 +109,9 @@
   </si>
   <si>
     <t xml:space="preserve">Sampling of continuous signals </t>
+  </si>
+  <si>
+    <t xml:space="preserve">x (70%)</t>
   </si>
   <si>
     <t xml:space="preserve">Mangler siste oppgave</t>
@@ -134,7 +128,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.00%"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -194,6 +188,11 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -585,6 +584,119 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="absolute">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>535680</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>511560</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>82800</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="1" name="Text Frame 1"/>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9006480" y="2884320"/>
+          <a:ext cx="2916720" cy="1797120"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="ffbf00"/>
+        </a:solidFill>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr lIns="0" rIns="0" tIns="0" bIns="0" anchor="t">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:p>
+          <a:r>
+            <a:rPr b="0" lang="nb-NO" sz="1200" strike="noStrike" u="none">
+              <a:effectLst/>
+              <a:uFillTx/>
+              <a:latin typeface="Times New Roman"/>
+            </a:rPr>
+            <a:t>Ting jeg kanskje burde se mer på:</a:t>
+          </a:r>
+          <a:endParaRPr b="0" lang="nb-NO" sz="1200" strike="noStrike" u="none">
+            <a:effectLst/>
+            <a:uFillTx/>
+            <a:latin typeface="Times New Roman"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:endParaRPr b="0" lang="nb-NO" sz="1200" strike="noStrike" u="none">
+            <a:effectLst/>
+            <a:uFillTx/>
+            <a:latin typeface="Times New Roman"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr b="0" lang="nb-NO" sz="1200" strike="noStrike" u="none">
+              <a:effectLst/>
+              <a:uFillTx/>
+              <a:latin typeface="Times New Roman"/>
+            </a:rPr>
+            <a:t>* De ulike DTFT/Z-transform egenskapene</a:t>
+          </a:r>
+          <a:endParaRPr b="0" lang="nb-NO" sz="1200" strike="noStrike" u="none">
+            <a:effectLst/>
+            <a:uFillTx/>
+            <a:latin typeface="Times New Roman"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr b="0" lang="nb-NO" sz="1200" strike="noStrike" u="none">
+              <a:effectLst/>
+              <a:uFillTx/>
+              <a:latin typeface="Times New Roman"/>
+            </a:rPr>
+            <a:t>	</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr b="0" lang="nb-NO" sz="1200" strike="noStrike" u="none">
+              <a:effectLst/>
+              <a:uFillTx/>
+              <a:latin typeface="Times New Roman"/>
+            </a:rPr>
+            <a:t>* Folding, time-shift etc</a:t>
+          </a:r>
+          <a:endParaRPr b="0" lang="nb-NO" sz="1200" strike="noStrike" u="none">
+            <a:effectLst/>
+            <a:uFillTx/>
+            <a:latin typeface="Times New Roman"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:endParaRPr b="0" lang="nb-NO" sz="1200" strike="noStrike" u="none">
+            <a:effectLst/>
+            <a:uFillTx/>
+            <a:latin typeface="Times New Roman"/>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -904,7 +1016,7 @@
         <v>9</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>10</v>
@@ -933,13 +1045,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>9</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="E5" s="1" t="n">
         <v>6</v>
@@ -968,16 +1080,16 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>8</v>
       </c>
       <c r="G6" s="14" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I6" s="15"/>
       <c r="J6" s="16"/>
@@ -1003,10 +1115,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="39.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1014,19 +1126,19 @@
         <v>7</v>
       </c>
       <c r="B8" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="G8" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="I8" s="19" t="s">
         <v>27</v>
-      </c>
-      <c r="G8" s="14" t="s">
-        <v>28</v>
-      </c>
-      <c r="I8" s="19" t="s">
-        <v>29</v>
       </c>
       <c r="J8" s="20"/>
       <c r="K8" s="21" t="n">
@@ -1039,17 +1151,17 @@
         <v>8</v>
       </c>
       <c r="B9" s="22" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C9" s="22"/>
       <c r="D9" s="23" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>8</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I9" s="24"/>
       <c r="J9" s="25"/>
@@ -1060,7 +1172,7 @@
         <v>9</v>
       </c>
       <c r="I10" s="27" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J10" s="28"/>
       <c r="K10" s="29"/>
@@ -1096,5 +1208,6 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>